<commit_message>
Fix chart rendering and add user-audit test suite.
Charts now scale axes correctly, clip to the plot area, use per-category colors with legends, and stay within the viewport. Demo workbook and user-audit cover VLOOKUP, sort, and end-to-end scenarios.
</commit_message>
<xml_diff>
--- a/demo/Arbuz-feature-demo.xlsx
+++ b/demo/Arbuz-feature-demo.xlsx
@@ -15,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="13">
+  <fonts count="16">
     <font/>
     <font>
       <color rgb="FF334155"/>
@@ -28,6 +28,16 @@
       <b/>
     </font>
     <font/>
+    <font>
+      <color rgb="FFB4222E"/>
+    </font>
+    <font/>
+    <font/>
+    <font/>
+    <font>
+      <i/>
+    </font>
+    <font/>
     <font/>
     <font/>
     <font>
@@ -35,11 +45,8 @@
     </font>
     <font/>
     <font/>
-    <font/>
-    <font/>
-    <font/>
   </fonts>
-  <fills count="15">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -58,18 +65,6 @@
       </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF3CD"/>
       </patternFill>
@@ -84,6 +79,29 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD4EDDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
@@ -92,7 +110,43 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="16">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -153,26 +207,8 @@
       <top/>
       <bottom/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-    </border>
   </borders>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment/>
     </xf>
@@ -182,38 +218,55 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="4" fontId="3" fillId="5" borderId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment/>
     </xf>
-    <xf numFmtId="4" fontId="7" fillId="9" borderId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment/>
     </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="14" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="15" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
 </styleSheet>
+</file>
+
+<file path=xl/arbuz/charts.xml><?xml version="1.0" encoding="utf-8"?>
+<arbuzCharts>
+  <sheet name="Charts">
+    <chart type="column" r1="0" c1="0" r2="5" c2="1" x="170" y="30" w="340" h="250" header="1" legend="1" title="Продажи (демо)"/>
+  </sheet>
+</arbuzCharts>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -236,26 +289,26 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Открытие и сохранение xlsx</t>
+        </is>
+      </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Файл → Сохранить как… → снова открыть этот файл</t>
         </is>
       </c>
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Открытие и сохранение xlsx</t>
-        </is>
-      </c>
     </row>
     <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Несколько листов</t>
+        </is>
+      </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Вкладки внизу: Formulas, Formats, Data…</t>
-        </is>
-      </c>
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Несколько листов</t>
         </is>
       </c>
     </row>
@@ -272,38 +325,38 @@
       </c>
     </row>
     <row r="5">
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Formulas: 1,5 и 25%</t>
+        </is>
+      </c>
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Десятичная запятая и %</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Formulas: 1,5 и 25%</t>
-        </is>
-      </c>
     </row>
     <row r="6">
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Лист Cross и Formulas!B2</t>
+        </is>
+      </c>
       <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Кросс-листовые формулы</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Лист Cross и Formulas!B2</t>
-        </is>
-      </c>
     </row>
     <row r="7">
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Formats → выделить A14:D16 → Ctrl+C / Ctrl+V</t>
+        </is>
+      </c>
       <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Копировать / вставить со стилями</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>Formats → выделить A2:D4 → Ctrl+C / Ctrl+V</t>
         </is>
       </c>
     </row>
@@ -344,38 +397,38 @@
       </c>
     </row>
     <row r="11">
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Data → выделить A1:D7 → Вид → Автофильтр → Фильтр столбца</t>
+        </is>
+      </c>
       <c r="A11" s="1" t="inlineStr">
         <is>
           <t>AutoFilter</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>Data → выделить A1:D7 → Вид → Автофильтр → Фильтр столбца</t>
-        </is>
-      </c>
     </row>
     <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Сортировка</t>
+        </is>
+      </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
           <t>Data → выделить таблицу → Вид → Sort A→Z</t>
         </is>
       </c>
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Сортировка</t>
-        </is>
-      </c>
     </row>
     <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Merge / Freeze</t>
+        </is>
+      </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Layout: merge B2:C2; Вид → Закрепить</t>
-        </is>
-      </c>
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>Merge / Freeze</t>
         </is>
       </c>
     </row>
@@ -404,14 +457,14 @@
       </c>
     </row>
     <row r="16">
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>Ctrl+P на листе Layout</t>
+        </is>
+      </c>
       <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Печать</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>Ctrl+P на листе Layout</t>
         </is>
       </c>
     </row>
@@ -458,88 +511,88 @@
           <t>D</t>
         </is>
       </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
     </row>
     <row r="2">
+      <c r="D2">
+        <f>TODAY()</f>
+      </c>
+      <c r="C2">
+        <f>Formulas!A2*10</f>
+      </c>
+      <c r="A2" t="n">
+        <v>1.5</v>
+      </c>
       <c r="B2" t="n">
         <v>0.25</v>
-      </c>
-      <c r="A2" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C2">
-        <f>Formulas!A2*10</f>
-      </c>
-      <c r="D2">
-        <f>TODAY()</f>
       </c>
     </row>
     <row r="3">
       <c r="C3">
         <f>IF(A2&gt;1;"да";"нет")</f>
       </c>
+      <c r="D3">
+        <f>AVERAGE(A2:A3)</f>
+      </c>
+      <c r="A3" t="n">
+        <v>2.5</v>
+      </c>
       <c r="B3">
         <f>A2*2</f>
       </c>
-      <c r="D3">
-        <f>AVERAGE(A2:A3)</f>
-      </c>
-      <c r="A3" t="n">
-        <v>2.5</v>
-      </c>
     </row>
     <row r="4">
+      <c r="A4">
+        <f>SUM(A2:A3)</f>
+      </c>
       <c r="C4">
         <f>VLOOKUP("яблоко";E5:F7;2;0)</f>
       </c>
-      <c r="A4">
-        <f>SUM(A2:A3)</f>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>цена</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>товар</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>цена</t>
-        </is>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="F6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>яблоко</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="F7" t="n">
+        <v>40</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>груша</t>
         </is>
-      </c>
-      <c r="B7" t="n">
-        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -584,31 +637,21 @@
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="3" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Жирный / курсив / цвета</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Жирный</t>
         </is>
       </c>
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Жирный / курсив / цвета</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>R2C2</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>R2C1</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>R2C3</t>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Курсив</t>
         </is>
       </c>
       <c r="A3" s="1" t="inlineStr">
@@ -618,63 +661,33 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>R3C2</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>R3C1</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>R3C3</t>
-        </is>
-      </c>
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>R3C0</t>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Красный текст</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>R4C3</t>
-        </is>
-      </c>
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>R4C0</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>R4C2</t>
-        </is>
-      </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>R4C1</t>
+          <t>Заливка</t>
         </is>
       </c>
     </row>
     <row r="6">
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Границы</t>
+        </is>
+      </c>
       <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Границы / перенос</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Границы</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Длинный текст с переносом на несколько строк в одной ячейке</t>
         </is>
@@ -691,23 +704,89 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="10" t="n">
         <v>1999.9</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="14" t="n">
         <v>42.5</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="11" t="n">
         <v>99.99</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>R13C0</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>R13C1</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>R13C3</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>R13C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>R14C3</t>
+        </is>
+      </c>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>R14C0</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>R14C1</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>R14C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>R15C1</t>
+        </is>
+      </c>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>R15C0</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>R15C3</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>R15C2</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -723,49 +802,44 @@
           <t>Цена</t>
         </is>
       </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Товар</t>
+        </is>
+      </c>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Отдел</t>
+        </is>
+      </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Товар</t>
-        </is>
-      </c>
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Отдел</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Яблоки</t>
-        </is>
-      </c>
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Склад</t>
-        </is>
+      <c r="D2" t="n">
+        <v>50</v>
       </c>
       <c r="C2" t="n">
         <v>12</v>
       </c>
-      <c r="D2" t="n">
-        <v>50</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Склад</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Яблоки</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="C3" t="n">
         <v>8</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Груши</t>
-        </is>
-      </c>
       <c r="D3" t="n">
         <v>40</v>
       </c>
@@ -774,48 +848,51 @@
           <t>Склад</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Груши</t>
+        </is>
+      </c>
     </row>
     <row r="4">
+      <c r="D4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Яблоки</t>
+        </is>
+      </c>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Магазин</t>
+        </is>
+      </c>
       <c r="C4" t="n">
         <v>5</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Яблоки</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>55</v>
-      </c>
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Магазин</t>
-        </is>
       </c>
     </row>
     <row r="5">
       <c r="D5" t="n">
         <v>70</v>
       </c>
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Магазин</t>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Сливы</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Сливы</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Магазин</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Склад</t>
-        </is>
+      <c r="D6" t="n">
+        <v>10</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
@@ -825,8 +902,10 @@
           <t>REPLACE_ME</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>10</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Склад</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -861,23 +940,23 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Янв</t>
+        </is>
+      </c>
       <c r="B2" t="n">
         <v>120</v>
       </c>
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Янв</t>
-        </is>
-      </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Фев</t>
+        </is>
+      </c>
       <c r="B3" t="n">
         <v>150</v>
-      </c>
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Фев</t>
-        </is>
       </c>
     </row>
     <row r="4">
@@ -891,23 +970,23 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Апр</t>
-        </is>
-      </c>
       <c r="B5" t="n">
         <v>180</v>
       </c>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Апр</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Май</t>
-        </is>
-      </c>
       <c r="B6" t="n">
         <v>140</v>
+      </c>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Май</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -963,98 +1042,98 @@
   </cols>
   <sheetData>
     <row r="1">
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Заголовок</t>
+        </is>
+      </c>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Заголовок</t>
-        </is>
-      </c>
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="24.00" customHeight="1">
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>Объединено B2:C2</t>
-        </is>
+      <c r="C2" t="n">
+        <v>10</v>
       </c>
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
-        <v>10</v>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Объединено B2:C2</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="C3" t="n">
         <v>20</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Строка 2</t>
-        </is>
-      </c>
       <c r="A3" t="n">
         <v>2</v>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Строка 2</t>
+        </is>
+      </c>
     </row>
     <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Строка 3</t>
+        </is>
+      </c>
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
       <c r="C4" t="n">
         <v>30</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Строка 3</t>
-        </is>
-      </c>
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Строка 4</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>40</v>
+      </c>
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="n">
-        <v>40</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Строка 4</t>
-        </is>
-      </c>
     </row>
     <row r="6">
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Строка 5</t>
+        </is>
+      </c>
       <c r="A6" t="n">
         <v>5</v>
-      </c>
-      <c r="C6" t="n">
-        <v>50</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Строка 5</t>
-        </is>
       </c>
     </row>
     <row r="7">
       <c r="C7" t="n">
         <v>60</v>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Строка 6</t>
+        </is>
+      </c>
       <c r="A7" t="n">
         <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Строка 6</t>
-        </is>
       </c>
     </row>
     <row r="8">
@@ -1076,11 +1155,11 @@
           <t>Строка 8</t>
         </is>
       </c>
+      <c r="C9" t="n">
+        <v>80</v>
+      </c>
       <c r="A9" t="n">
         <v>8</v>
-      </c>
-      <c r="C9" t="n">
-        <v>80</v>
       </c>
     </row>
     <row r="10">
@@ -1100,39 +1179,39 @@
       <c r="C11" t="n">
         <v>100</v>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Строка 10</t>
+        </is>
+      </c>
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Строка 10</t>
-        </is>
-      </c>
     </row>
     <row r="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Строка 11</t>
-        </is>
+      <c r="A12" t="n">
+        <v>11</v>
       </c>
       <c r="C12" t="n">
         <v>110</v>
       </c>
-      <c r="A12" t="n">
-        <v>11</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Строка 11</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="C13" t="n">
         <v>120</v>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Строка 12</t>
-        </is>
-      </c>
       <c r="A13" t="n">
         <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Строка 12</t>
+        </is>
       </c>
     </row>
     <row r="15">

</xml_diff>